<commit_message>
chore: update chauffeur config xlsx with homeCity and depot for all drivers
Adds city/depot mappings for 15 drivers including Tayeb (Lebbeke / Albert I),
Bendada (Liège / Hoeselt), Allouchi (Quevaucamps / Roeselare), etc.
Required for commute exclusion logic in WebfleetImport.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/Chauffeur M-D LOG.xlsx
+++ b/samples/Chauffeur M-D LOG.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/901be47c64b9ecc4/Bureau/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="201" documentId="8_{F8062516-CD78-4A3F-82A8-6932A2B46C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BE1E94D-1503-4522-A15C-EAB2CFBDF083}"/>
+  <xr:revisionPtr revIDLastSave="216" documentId="8_{F8062516-CD78-4A3F-82A8-6932A2B46C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0306E71-00A0-4CAB-A3AF-38B990914F17}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="10" activeTab="13" xr2:uid="{64FEA768-FFDD-4D4D-AF34-7983E5A84874}"/>
+    <workbookView xWindow="28692" yWindow="-108" windowWidth="29016" windowHeight="15696" firstSheet="10" activeTab="14" xr2:uid="{64FEA768-FFDD-4D4D-AF34-7983E5A84874}"/>
   </bookViews>
   <sheets>
     <sheet name="ADIB ABDERAZAK" sheetId="1" r:id="rId1"/>
@@ -27,6 +27,7 @@
     <sheet name="SIDIBE SIDIBE Mohamed" sheetId="12" r:id="rId12"/>
     <sheet name="TEMSAMANI JAWAD" sheetId="13" r:id="rId13"/>
     <sheet name="YOUSFI FOUAD" sheetId="14" r:id="rId14"/>
+    <sheet name="BOUHTALA OUCHEN HAMID " sheetId="15" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="107">
   <si>
     <t>ADIB ABDERAZAK</t>
   </si>
@@ -360,13 +361,28 @@
   </si>
   <si>
     <t>Tournée distribution ou Diegem Wilrijk - Diegem</t>
+  </si>
+  <si>
+    <t>HAMID</t>
+  </si>
+  <si>
+    <t>BOUHTALA OUCHEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Groeningerplein 23 bus 201, </t>
+  </si>
+  <si>
+    <t>2140 Borgherhout Antwerpen</t>
+  </si>
+  <si>
+    <t>Départ albertlaan, retour albertlaan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -400,6 +416,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -421,7 +443,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -430,9 +452,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1065,16 +1088,16 @@
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="6"/>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
@@ -1208,6 +1231,129 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98B77BED-1575-49CD-8A7A-24195C599AD8}">
+  <dimension ref="A2:C21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="5"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="5"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="5"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="5"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="5"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="5"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="5"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93ADFE5E-773A-479B-A4FF-23DA7A819C20}">
   <dimension ref="A2:B17"/>
@@ -1232,7 +1378,7 @@
       <c r="A11" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1347,7 +1493,7 @@
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
+      <c r="A27" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1545,7 +1691,7 @@
       <c r="A18" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1553,7 +1699,7 @@
       <c r="A19" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1739,13 +1885,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>79</v>
       </c>
-      <c r="B18" s="5"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>42</v>
       </c>

</xml_diff>